<commit_message>
feat: atualização painel de notícias, feriados no FullCalendar e botão de submissão em Eventos
</commit_message>
<xml_diff>
--- a/api/data/examples/eventos.xlsx
+++ b/api/data/examples/eventos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bibianadibellacostabatista/Documents/Thais/Igen/intranet-pasta/projeto-intranet/api/data/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A5E7198-5F64-B943-8D86-89F435E8F10F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{440643C0-6D16-5C4D-A654-A45E9B73538A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="1000" windowWidth="27840" windowHeight="16340" xr2:uid="{6201E4D8-F5B0-AA41-9DF5-65B9990920B6}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Data</t>
   </si>
@@ -75,16 +75,27 @@
   </si>
   <si>
     <t>Submissão</t>
+  </si>
+  <si>
+    <t>https://www.atcmeeting.org/Learn/Calls-for-Content/Abstract-Program</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -107,14 +118,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -454,6 +468,7 @@
     <col min="2" max="2" width="44.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="60.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
@@ -497,11 +512,18 @@
       <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="2" t="s">
         <v>11</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D3" r:id="rId1" xr:uid="{0D282B20-E8C3-BB4D-9210-E0C7086500AC}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{160BF433-F5C2-4547-AD71-A7D9072E1623}"/>
+  </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>